<commit_message>
Report Suite Fabian-review: deliverables + regenerated import/id-map (498 cases)
COVERAGE-REDERIVATION (9 Loom items verdicted both directions + surface matrix),
CASES-CREATED (18 new + 1 updated with links), completion report, outstanding
register (RS-FB1..5). Regenerated import + id-map re-merged from live: four counts
set-equal both ways (live 498 / local 498 / id-map 498 / import 498), 0 blanks,
shredding guard PASSED, header sha256 == peers. Foreign 12 untouched. Run-359
sync NOT executed (needs per-ask auth).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Parts-Velocity-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Parts-Velocity-Report_testrail-import.xlsx
@@ -1503,6 +1503,10 @@
 4. A user who can reach only one location never sees the column at all.
 5. Whenever the column is shown on screen, both downloads include it in the same position (leftmost, before Type), with the same values — each inventory row's own location, and "Multiple" on the merged Special Order row.
 Note for the tester: two points about this column are still unsettled for Parts Velocity, and the product owner has been asked. One is whether narrowing the location selection hides it; the other is whether it can be switched off in the column picker and whether it counts toward the fourteen default columns. Whatever you see on those two points, do not raise a bug and do not fail the test for them — record what you see and carry on. The question is here: https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/questions-2026-08-06/Questions-for-Chris-Ward_Report-Suite_2026-08-11.xlsx
+What you should see today: the Location column is not the leftmost column. It sits sixth, after Vendor, in all three places - on screen and in both downloads. The values themselves are right, including "Multiple" on the merged Special Order row. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8938
+- If you see exactly that, mark this test FAILED and do not raise anything new.
+- If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
+- If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
 This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Parts Velocity report specification version 6 (S2-R12, S3-R10, S7-R8, S6-R11), read on 11 August 2026. That specification still says two different things about this column: S3-R10 was rewritten in version 6 to make it access-gated and toggleable in the column picker, while S2-R12 still ties it to the current location scope and S4-R2/S4-R3 list twenty picker columns that do not include it. Chris Ward has been asked which is right, so neither reading is asserted here.
 Last checked against build v3.5-16cf83f on 8/6/2026.

</xml_diff>